<commit_message>
Sync October 9 team records, rankings and province statistics
</commit_message>
<xml_diff>
--- a/data/team-checklist.xlsx
+++ b/data/team-checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R51431e5499114ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R3a55688b106544f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -358,7 +358,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>2026-09-28 新疆鸟会队大年记录</x:v>
+        <x:v>2026-10-09 新疆鸟会队大年记录</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -370,8 +370,8 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:f>"共记录 "&amp;COUNTIF(H6:H1523,"已记录")&amp;" 种 / 名录 "&amp;COUNTA(C6:C1523)&amp;" 种；全国第 55 名。浅绿色为队伍已记录。"</x:f>
-        <x:v>共记录 958 种 / 名录 1518 种；全国第 55 名。浅绿色为队伍已记录。</x:v>
+        <x:f>"共记录 "&amp;COUNTIF(H6:H1523,"已记录")&amp;" 种 / 名录 "&amp;COUNTA(C6:C1523)&amp;" 种；全国第 60 名。浅绿色为队伍已记录。"</x:f>
+        <x:v>共记录 958 种 / 名录 1518 种；全国第 60 名。浅绿色为队伍已记录。</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -383,7 +383,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>更新时间 2026-09-28 16:02:13；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
+        <x:v>更新时间 2026-10-09 03:01:24；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>

</xml_diff>

<commit_message>
Sync October 10 team records and statistics
</commit_message>
<xml_diff>
--- a/data/team-checklist.xlsx
+++ b/data/team-checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R3a55688b106544f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R18da3f4cde424178"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -358,7 +358,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>2026-10-09 新疆鸟会队大年记录</x:v>
+        <x:v>2026-10-10 新疆鸟会队大年记录</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -383,7 +383,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>更新时间 2026-10-09 03:01:24；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
+        <x:v>更新时间 2026-10-10 00:02:22；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>

</xml_diff>

<commit_message>
Sync October 12 team records and statistics
</commit_message>
<xml_diff>
--- a/data/team-checklist.xlsx
+++ b/data/team-checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R18da3f4cde424178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="Ra08009f5f3ab49cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -87,7 +87,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -358,7 +364,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>2026-10-10 新疆鸟会队大年记录</x:v>
+        <x:v>2026-10-12 新疆鸟会队大年记录</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -371,7 +377,7 @@
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:f>"共记录 "&amp;COUNTIF(H6:H1523,"已记录")&amp;" 种 / 名录 "&amp;COUNTA(C6:C1523)&amp;" 种；全国第 60 名。浅绿色为队伍已记录。"</x:f>
-        <x:v>共记录 958 种 / 名录 1518 种；全国第 60 名。浅绿色为队伍已记录。</x:v>
+        <x:v>共记录 959 种 / 名录 1518 种；全国第 60 名。浅绿色为队伍已记录。</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -383,7 +389,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>更新时间 2026-10-10 00:02:22；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
+        <x:v>更新时间 2026-10-12 11:08:04；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -15016,29 +15022,29 @@
       </x:c>
     </x:row>
     <x:row r="567" ht="34" customHeight="1">
-      <x:c r="A567" s="12" t="n">
+      <x:c r="A567" s="16" t="n">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="B567" s="3" t="str">
+      <x:c r="B567" s="17" t="str">
         <x:v>翠鸟科</x:v>
       </x:c>
-      <x:c r="C567" s="3" t="str">
+      <x:c r="C567" s="17" t="str">
         <x:v>赤翡翠</x:v>
       </x:c>
-      <x:c r="D567" s="11" t="str">
+      <x:c r="D567" s="18" t="str">
         <x:v>Halcyon coromanda</x:v>
       </x:c>
-      <x:c r="E567" s="3" t="str">
+      <x:c r="E567" s="17" t="str">
         <x:v>Ruddy Kingfisher</x:v>
       </x:c>
-      <x:c r="F567" s="12" t="str">
-        <x:v>LC</x:v>
-      </x:c>
-      <x:c r="G567" s="12" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="H567" s="12" t="str">
-        <x:v>未记录</x:v>
+      <x:c r="F567" s="16" t="str">
+        <x:v>LC</x:v>
+      </x:c>
+      <x:c r="G567" s="16" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="H567" s="16" t="str">
+        <x:v>已记录</x:v>
       </x:c>
     </x:row>
     <x:row r="568" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Sync October 13 team records and statistics
</commit_message>
<xml_diff>
--- a/data/team-checklist.xlsx
+++ b/data/team-checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="Ra08009f5f3ab49cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R39ee9a29124042f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -364,7 +364,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>2026-10-12 新疆鸟会队大年记录</x:v>
+        <x:v>2026-10-13 新疆鸟会队大年记录</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -389,7 +389,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>更新时间 2026-10-12 11:08:04；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
+        <x:v>更新时间 2026-10-13 01:04:43；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>

</xml_diff>

<commit_message>
Sync October 16 team records and statistics
</commit_message>
<xml_diff>
--- a/data/team-checklist.xlsx
+++ b/data/team-checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="R39ee9a29124042f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整记录清单" sheetId="1" r:id="Rb858fe2503884874"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -364,7 +364,7 @@
   <x:sheetData>
     <x:row r="1" ht="52" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>2026-10-13 新疆鸟会队大年记录</x:v>
+        <x:v>2026-10-16 新疆鸟会队大年记录</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -376,8 +376,8 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:f>"共记录 "&amp;COUNTIF(H6:H1523,"已记录")&amp;" 种 / 名录 "&amp;COUNTA(C6:C1523)&amp;" 种；全国第 60 名。浅绿色为队伍已记录。"</x:f>
-        <x:v>共记录 959 种 / 名录 1518 种；全国第 60 名。浅绿色为队伍已记录。</x:v>
+        <x:f>"共记录 "&amp;COUNTIF(H6:H1523,"已记录")&amp;" 种 / 名录 "&amp;COUNTA(C6:C1523)&amp;" 种；全国第 61 名。浅绿色为队伍已记录。"</x:f>
+        <x:v>共记录 960 种 / 名录 1518 种；全国第 61 名。浅绿色为队伍已记录。</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -389,7 +389,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>更新时间 2026-10-13 01:04:43；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
+        <x:v>更新时间 2026-10-16 04:02:03；记录来源：中国观鸟记录中心 https://www.birdreport.cn/；名录：中国鸟类名录 12.0＋队长调整。</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -13254,29 +13254,29 @@
       </x:c>
     </x:row>
     <x:row r="499" ht="34" customHeight="1">
-      <x:c r="A499" s="12" t="n">
+      <x:c r="A499" s="16" t="n">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="B499" s="3" t="str">
+      <x:c r="B499" s="17" t="str">
         <x:v>杜鹃科</x:v>
       </x:c>
-      <x:c r="C499" s="3" t="str">
+      <x:c r="C499" s="17" t="str">
         <x:v>北棕腹鹰鹃</x:v>
       </x:c>
-      <x:c r="D499" s="11" t="str">
+      <x:c r="D499" s="18" t="str">
         <x:v>Hierococcyx hyperythrus</x:v>
       </x:c>
-      <x:c r="E499" s="3" t="str">
+      <x:c r="E499" s="17" t="str">
         <x:v>Northern Hawk-Cuckoo</x:v>
       </x:c>
-      <x:c r="F499" s="12" t="str">
-        <x:v>LC</x:v>
-      </x:c>
-      <x:c r="G499" s="12" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="H499" s="12" t="str">
-        <x:v>未记录</x:v>
+      <x:c r="F499" s="16" t="str">
+        <x:v>LC</x:v>
+      </x:c>
+      <x:c r="G499" s="16" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="H499" s="16" t="str">
+        <x:v>已记录</x:v>
       </x:c>
     </x:row>
     <x:row r="500" ht="34" customHeight="1">

</xml_diff>